<commit_message>
Fill max body size
</commit_message>
<xml_diff>
--- a/Datos/Species traits - TDF.xlsx
+++ b/Datos/Species traits - TDF.xlsx
@@ -2282,7 +2282,9 @@
       <c r="F11" s="8">
         <v>1.45</v>
       </c>
-      <c r="G11" s="9"/>
+      <c r="G11" s="8">
+        <v>1.45</v>
+      </c>
       <c r="H11" t="s" s="7">
         <v>26</v>
       </c>
@@ -2364,7 +2366,9 @@
       <c r="F13" s="8">
         <v>0.045</v>
       </c>
-      <c r="G13" s="9"/>
+      <c r="G13" s="8">
+        <v>0.045</v>
+      </c>
       <c r="H13" t="s" s="7">
         <v>26</v>
       </c>
@@ -3384,7 +3388,9 @@
       <c r="F37" s="13">
         <v>1</v>
       </c>
-      <c r="G37" s="9"/>
+      <c r="G37" s="8">
+        <v>1</v>
+      </c>
       <c r="H37" t="s" s="7">
         <v>17</v>
       </c>
@@ -3422,7 +3428,9 @@
       <c r="F38" s="13">
         <v>0.2</v>
       </c>
-      <c r="G38" s="9"/>
+      <c r="G38" s="8">
+        <v>0.2</v>
+      </c>
       <c r="H38" t="s" s="7">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
Add fake carnivores to test model
</commit_message>
<xml_diff>
--- a/Datos/Species traits - TDF.xlsx
+++ b/Datos/Species traits - TDF.xlsx
@@ -178,7 +178,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="84">
   <si>
     <t>Class</t>
   </si>
@@ -414,6 +414,12 @@
     <t>Sterna_hirundinacea</t>
   </si>
   <si>
+    <t>Fake_carnivore1</t>
+  </si>
+  <si>
+    <t>Fake_carnivore2</t>
+  </si>
+  <si>
     <t>Mamíferos vivientes</t>
   </si>
   <si>
@@ -426,7 +432,7 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color indexed="11"/>
+        <color indexed="12"/>
         <rFont val="CloSans, &quot;CloSans override&quot;, &quot;Noto Sans&quot;, &quot;Noto Sans Hebrew&quot;, -apple-system, BlinkMacSystemFont, &quot;Segoe UI&quot;, Roboto, Oxygen-Sans, Ubuntu, Cantarell, &quot;Helvetica Neue&quot;, sans-serif"/>
       </rPr>
       <t>Birds of the World (G. M. Kirwan, Editor). Cornell Lab of Ornithology, Ithaca, NY, USA.</t>
@@ -474,24 +480,30 @@
     </font>
     <font>
       <sz val="9"/>
-      <color indexed="10"/>
+      <color indexed="11"/>
       <name val="&quot;Open Sans&quot;"/>
     </font>
     <font>
       <sz val="11"/>
-      <color indexed="11"/>
+      <color indexed="12"/>
       <name val="CloSans, &quot;CloSans override&quot;, &quot;Noto Sans&quot;, &quot;Noto Sans Hebrew&quot;, -apple-system, BlinkMacSystemFont, &quot;Segoe UI&quot;, Roboto, Oxygen-Sans, Ubuntu, Cantarell, &quot;Helvetica Neue&quot;, sans-serif"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -501,13 +513,13 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
         <color indexed="8"/>
@@ -516,57 +528,57 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
         <color indexed="8"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -580,41 +592,41 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
         <color indexed="8"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -623,10 +635,10 @@
         <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -641,10 +653,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -662,76 +685,76 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="5" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="5" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="6" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -751,6 +774,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
       <rgbColor rgb="ff414141"/>
       <rgbColor rgb="ff2e261f"/>
@@ -956,12 +980,12 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -993,10 +1017,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Arial"/>
-            <a:ea typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-            <a:sym typeface="Arial"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1235,12 +1259,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1544,10 +1568,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Arial"/>
-            <a:ea typeface="Arial"/>
-            <a:cs typeface="Arial"/>
-            <a:sym typeface="Arial"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -3422,7 +3446,7 @@
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
       <c r="D38" s="15"/>
-      <c r="E38" t="s" s="18">
+      <c r="E38" t="s" s="19">
         <v>77</v>
       </c>
       <c r="F38" s="13">
@@ -3456,14 +3480,22 @@
       <c r="AB38" s="9"/>
     </row>
     <row r="39" ht="13.65" customHeight="1">
-      <c r="A39" s="9"/>
+      <c r="A39" t="s" s="7">
+        <v>78</v>
+      </c>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
-      <c r="E39" s="19"/>
+      <c r="E39" t="s" s="7">
+        <v>78</v>
+      </c>
       <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
+      <c r="G39" s="8">
+        <v>5</v>
+      </c>
+      <c r="H39" t="s" s="7">
+        <v>47</v>
+      </c>
       <c r="I39" s="9"/>
       <c r="J39" s="9"/>
       <c r="K39" s="9"/>
@@ -3486,14 +3518,22 @@
       <c r="AB39" s="9"/>
     </row>
     <row r="40" ht="13.65" customHeight="1">
-      <c r="A40" s="9"/>
+      <c r="A40" t="s" s="7">
+        <v>79</v>
+      </c>
       <c r="B40" s="9"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
-      <c r="E40" s="9"/>
+      <c r="E40" t="s" s="7">
+        <v>79</v>
+      </c>
       <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
+      <c r="G40" s="8">
+        <v>500</v>
+      </c>
+      <c r="H40" t="s" s="7">
+        <v>47</v>
+      </c>
       <c r="I40" s="9"/>
       <c r="J40" s="9"/>
       <c r="K40" s="9"/>
@@ -32671,10 +32711,10 @@
   <sheetData>
     <row r="1" ht="14" customHeight="1">
       <c r="A1" t="s" s="21">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B1" t="s" s="22">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C1" s="23"/>
       <c r="D1" s="9"/>
@@ -32682,10 +32722,10 @@
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" t="s" s="24">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s" s="14">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>

</xml_diff>